<commit_message>
READMEs ueberarbeitet: Voraussetzungen praezisiert (Excel + Word), Text gestrafft
- Word-Abhaengigkeit der Projekte 1, 3, 4 jetzt ueberall klar benannt
- Braucht-Spalte in der Portfolio-Uebersicht ergaenzt
- Wiederholungen und Marketing-Floskeln entfernt

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_Eingangsrechnungen/output/Rechnungsuebersicht.xlsx
+++ b/01_Eingangsrechnungen/output/Rechnungsuebersicht.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\.Clode\.Clode_Cloude\портфолио\01_Eingangsrechnungen\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41097519-89AB-48AD-B7D1-EC057782F462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4F4AEB2-E9E4-4743-8FFC-041C20B3B03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11505" xr2:uid="{CD9D74F2-F53A-4F56-9FB4-2336C5696FEF}"/>
+    <workbookView xWindow="4305" yWindow="2805" windowWidth="21600" windowHeight="11505" xr2:uid="{23CE6776-570E-47BA-80A9-E2A64838BE0A}"/>
   </bookViews>
   <sheets>
     <sheet name="Eingangsrechnungen" sheetId="1" r:id="rId1"/>
@@ -577,7 +577,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1566142C-3867-4EC1-8646-67170748CCF3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E0146ED-6289-45EF-BB82-794621F8D047}">
   <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -909,7 +909,7 @@
       <c r="I12" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I10" xr:uid="{1566142C-3867-4EC1-8646-67170748CCF3}"/>
+  <autoFilter ref="A1:I10" xr:uid="{4E0146ED-6289-45EF-BB82-794621F8D047}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>